<commit_message>
Implement item selling functionality and enhance player inventory management
- Added a `sell_item` function to facilitate item sales in the shop, including inventory updates and currency adjustments.
- Updated the `Player` class to reflect changes in inventory and currency after item sales.
- Enhanced the UI to provide feedback on successful sales and current inventory status.
- Modified the shop interface to display available items for sale and their respective prices.
- Updated tests to ensure the correct functionality of the new selling logic and its integration with the inventory system.
</commit_message>
<xml_diff>
--- a/item_types.xlsx
+++ b/item_types.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\info\Documents\Projects\dungeon-console\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_C4C2AE743F73477F8C6234DF1CC34D96802312FB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{077657A5-9031-43D2-BCF4-8C3E67DF6544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Items" sheetId="1" r:id="rId1"/>
@@ -18,10 +18,9 @@
     <sheet name="Field reference" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Items!$A$1:$E$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Items!$A$1:$E$42</definedName>
   </definedNames>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -106,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="51">
   <si>
     <t>item_id</t>
   </si>
@@ -250,6 +249,15 @@
   </si>
   <si>
     <t>Blank = default sprite path</t>
+  </si>
+  <si>
+    <t>candle</t>
+  </si>
+  <si>
+    <t>Candle</t>
+  </si>
+  <si>
+    <t>Generates a small amount of light</t>
   </si>
 </sst>
 </file>
@@ -645,7 +653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -682,7 +690,7 @@
         <v>7</v>
       </c>
       <c r="D2" s="2">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>8</v>
@@ -690,78 +698,86 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="D3" s="2">
-        <v>5</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>12</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D4" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D5" s="2">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="2">
+        <v>15</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D7" s="2">
         <v>20</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
@@ -1001,8 +1017,15 @@
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
     </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="3"/>
+      <c r="B42" s="3"/>
+      <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E41" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:E42" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor combat mechanics for improved player experience
- Adjusted monster spawn rates in `map_generator.py` to enhance encounter dynamics.
- Implemented aggressive monster behavior in `monster_ai.py`, allowing them to engage in ongoing player combat.
- Updated `CombatSystem` to indicate whether player actions consume turns, streamlining combat flow in `combat.py`.
- Improved turn registration and state updates in `dungeon_crawler.py` for better combat action handling.
- Added tests to ensure the reliability of new monster behaviors and combat interactions.
</commit_message>
<xml_diff>
--- a/item_types.xlsx
+++ b/item_types.xlsx
@@ -635,7 +635,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>A wooden torch. Light it in the dungeon for steady light (sight 3). Burns for about 1000 turns.</t>
+          <t>A wooden torch. Light it in the dungeon for steady light (sight 20). Burns for about 1000 turns.</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>1000</v>
@@ -1066,9 +1066,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1111,9 +1109,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>

</xml_diff>